<commit_message>
Name the work in the opener only for a single print
A pair or a quartet is just the edition phrase ("a quartet of new limited
edition prints"), and the hook that follows names the work; many sets have no
collective name anyway. Untitled works from a named series keep "from the
Dream House series". Same rule in the workbook and the template; the Rules
sheet says so.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KCpXfXvgVaMZkSdhMYLgwy
</commit_message>
<xml_diff>
--- a/tool/release-copy-aiweiwei-embroidery-tl-26.xlsx
+++ b/tool/release-copy-aiweiwei-embroidery-tl-26.xlsx
@@ -1131,7 +1131,7 @@
         </is>
       </c>
       <c r="B47" s="10">
-        <f>IF($B$12="yes",$B$13&amp;" from the "&amp;$B$11&amp;" series",$B$11&amp;", "&amp;$B$13)</f>
+        <f>IF($B$12="yes",$B$13&amp;" from the "&amp;$B$11&amp;" series",IF($B$14=1,$B$11&amp;", "&amp;$B$13,$B$13))</f>
         <v/>
       </c>
     </row>
@@ -4521,7 +4521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4598,130 +4598,142 @@
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Fragments</t>
+          <t>Naming the work</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>Four per release, written once: bio (2 to 3 sentences, Coming Soon only), hook (1 to 2 sentences about the work, in every post and email), making (one sentence on how it was made), quote (verbatim). The hook and bio must not repeat each other.</t>
+          <t>The opener names the work only for a single print: 'The Changeling, a new limited edition print'. A pair or a quartet is just the edition phrase, and the hook names the work; many sets have no collective name anyway. Untitled works from a named series read 'six new limited edition prints from the Dream House series'.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Voice</t>
+          <t>Fragments</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Fragments are voice-neutral: no we or our, no artist name in the hook or the making line, and 'printmakers at Make-Ready' where it applies. The sheet adds 'our'. The Insiders email and the first-time survey are signed by the advisor named on Inputs. Features never say 'our'.</t>
+          <t>Four per release, written once: bio (2 to 3 sentences, Coming Soon only), hook (1 to 2 sentences about the work, in every post and email), making (one sentence on how it was made), quote (verbatim). The hook and bio must not repeat each other.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>Who and what</t>
+          <t>Voice</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>'by {artist}' is always the artist. 'collaboration with {collab_with}' is the artist's name, or the estate. 'unit' is what one is called (print, embroidery, sculpture), and the sheet writes 'a print' or 'an embroidery' wherever a line names one.</t>
+          <t>Fragments are voice-neutral: no we or our, no artist name in the hook or the making line, and 'printmakers at Make-Ready' where it applies. The sheet adds 'our'. The Insiders email and the first-time survey are signed by the advisor named on Inputs. Features never say 'our'.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>Features</t>
+          <t>Who and what</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>The standard three (signed by the artist, individually numbered, free worldwide shipping) plus anything bespoke: framed, a set offer, a partner credit. One line of short sentences in a post, a list in an email. The beneficiary follows, named once.</t>
+          <t>'by {artist}' is always the artist. 'collaboration with {collab_with}' is the artist's name, or the estate. 'unit' is what one is called (print, embroidery, sculpture), and the sheet writes 'a print' or 'an embroidery' wherever a line names one.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>Beneficiary</t>
+          <t>Features</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>One phrase everywhere: 'released in support of'. It goes in the opener unless the hook already names the beneficiary.</t>
+          <t>The standard three (signed by the artist, individually numbered, free worldwide shipping) plus anything bespoke: framed, a set offer, a partner credit. One line of short sentences in a post, a list in an email. The beneficiary follows, named once.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>Framing offer</t>
+          <t>Beneficiary</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>A framing code on Inputs adds the first-purchase framing line to Early Access, Now Live, 3 days to go and Last chance. Blank means no offer.</t>
+          <t>One phrase everywhere: 'released in support of'. It goes in the opener unless the hook already names the beneficiary.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>Action lines</t>
+          <t>Framing offer</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Three CTAs: get updates before launch, enter the draw for a draw, buy one for an open window. One deadline form: Closes {date} at {time} UK time, or 'until {time} on {weekday}, {date}' in an email.</t>
+          <t>A framing code on Inputs adds the first-purchase framing line to Early Access, Now Live, 3 days to go and Last chance. Blank means no offer.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>Mechanic and window</t>
+          <t>Action lines</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Set mechanic to timed or draw and the sheet switches every line. For a timed edition, a 48-hour window gets the halfway email; a one-week window gets 5 days to go and 3 days to go.</t>
+          <t>Three CTAs: get updates before launch, enter the draw for a draw, buy one for an open window. One deadline form: Closes {date} at {time} UK time, or 'until {time} on {weekday}, {date}' in an email.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>Dates</t>
+          <t>Mechanic and window</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>Enter launch and close once as date and time; the sheet derives '30 April', '14:00 UK time', 'Thursday' and '07 May' where each email needs them.</t>
+          <t>Set mechanic to timed or draw and the sheet switches every line. For a timed edition, a 48-hour window gets the halfway email; a one-week window gets 5 days to go and 3 days to go.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>What stays written</t>
+          <t>Dates</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>A delay reason, a framing paragraph, editorial deep dives, the rest of the Monthly Preview, the artist's own email, artist-local times, and anything for a second release.</t>
+          <t>Enter launch and close once as date and time; the sheet derives '30 April', '14:00 UK time', 'Thursday' and '07 May' where each email needs them.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="12" t="inlineStr">
         <is>
+          <t>What stays written</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>A delay reason, a framing paragraph, editorial deep dives, the rest of the Monthly Preview, the artist's own email, artist-local times, and anything for a second release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="46" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
           <t>How to use</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>Fill the blue cells on Inputs. Read Posts, Tweets and Emails. To change the house wording, edit the blue cells on Lines once.</t>
         </is>

</xml_diff>

<commit_message>
Add the qualifier: the written tail of the email opener
The opener's tail is now the title (single print only), the edition phrase,
and a qualifier written for the release: "spanning five decades of the
artist's career", "from his iconic Dream House series", ", offered
individually, in pairs or as a complete quartet". The same tail serves the
Insiders email, LE early access, Now Live and the Monthly Preview paragraph.
The series special case goes; a qualifier says it. The validator holds the
qualifier to ten words, a phrase not a sentence, no we or our, no artist
name, no beneficiary.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KCpXfXvgVaMZkSdhMYLgwy
</commit_message>
<xml_diff>
--- a/tool/release-copy-aiweiwei-embroidery-tl-26.xlsx
+++ b/tool/release-copy-aiweiwei-embroidery-tl-26.xlsx
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -999,425 +999,442 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="48" customHeight="1">
+    <row r="35" ht="32" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
         <is>
+          <t>qualifier</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>, offered individually, in pairs or as a complete quartet</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>a few words after the edition phrase in the email opener, e.g. spanning five decades of the artist's career. Ten words at most, a phrase not a sentence, no we or our, no artist name, no beneficiary. Blank for none.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="48" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
           <t>making</t>
         </is>
       </c>
-      <c r="B35" s="8" t="inlineStr">
+      <c r="B36" s="8" t="inlineStr">
         <is>
           <t>Each embroidery was produced in close collaboration with the artist, translating the pixelated texture and bold presence of the original toy brick works into approximately 460,000 stitches.</t>
         </is>
       </c>
-      <c r="C35" s="9" t="inlineStr">
+      <c r="C36" s="9" t="inlineStr">
         <is>
           <t>one sentence on how the edition was made; write 'printmakers at Make-Ready' and the sheet adds 'our'.</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="32" customHeight="1">
-      <c r="A36" s="4" t="inlineStr">
+    <row r="37" ht="32" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>quote</t>
         </is>
       </c>
-      <c r="B36" s="8" t="inlineStr"/>
-      <c r="C36" s="9" t="inlineStr">
+      <c r="B37" s="8" t="inlineStr"/>
+      <c r="C37" s="9" t="inlineStr">
         <is>
           <t>verbatim, a complete sentence, or blank</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="7" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
         <is>
           <t>Derived (formulas, do not edit)</t>
         </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>named</t>
-        </is>
-      </c>
-      <c r="B39" s="10">
-        <f>$B$4&amp;IF($B$6="",""," (@"&amp;$B$6&amp;")")</f>
-        <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>named_x</t>
+          <t>named</t>
         </is>
       </c>
       <c r="B40" s="10">
-        <f>$B$4&amp;IF($B$7="",""," (@"&amp;$B$7&amp;")")</f>
+        <f>$B$4&amp;IF($B$6="",""," (@"&amp;$B$6&amp;")")</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>collab_x</t>
+          <t>named_x</t>
         </is>
       </c>
       <c r="B41" s="10">
-        <f>IF($B$5=$B$4,$B$40,$B$5)</f>
+        <f>$B$4&amp;IF($B$7="",""," (@"&amp;$B$7&amp;")")</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>a_unit</t>
+          <t>collab_x</t>
         </is>
       </c>
       <c r="B42" s="10">
-        <f>IF(OR(LEFT($B$15,1)="a",LEFT($B$15,1)="e",LEFT($B$15,1)="i",LEFT($B$15,1)="o",LEFT($B$15,1)="u"),"an ","a ")&amp;$B$15</f>
+        <f>IF($B$5=$B$4,$B$41,$B$5)</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>work</t>
+          <t>a_unit</t>
         </is>
       </c>
       <c r="B43" s="10">
-        <f>IF($B$12="yes","the "&amp;$B$11&amp;" series","‘"&amp;$B$11&amp;"’")</f>
+        <f>IF(OR(LEFT($B$15,1)="a",LEFT($B$15,1)="e",LEFT($B$15,1)="i",LEFT($B$15,1)="o",LEFT($B$15,1)="u"),"an ","a ")&amp;$B$15</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>Work</t>
+          <t>work</t>
         </is>
       </c>
       <c r="B44" s="10">
-        <f>UPPER(LEFT($B$43,1))&amp;MID($B$43,2,999)</f>
+        <f>IF($B$12="yes","the "&amp;$B$11&amp;" series","‘"&amp;$B$11&amp;"’")</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>work_email</t>
+          <t>Work</t>
         </is>
       </c>
       <c r="B45" s="10">
-        <f>IF($B$12="yes","the "&amp;$B$11&amp;" series",$B$11)</f>
+        <f>UPPER(LEFT($B$44,1))&amp;MID($B$44,2,999)</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>Work_email</t>
+          <t>work_email</t>
         </is>
       </c>
       <c r="B46" s="10">
-        <f>UPPER(LEFT($B$45,1))&amp;MID($B$45,2,999)</f>
+        <f>IF($B$12="yes","the "&amp;$B$11&amp;" series",$B$11)</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>work_intro</t>
+          <t>Work_email</t>
         </is>
       </c>
       <c r="B47" s="10">
-        <f>IF($B$12="yes",$B$13&amp;" from the "&amp;$B$11&amp;" series",IF($B$14=1,$B$11&amp;", "&amp;$B$13,$B$13))</f>
+        <f>UPPER(LEFT($B$46,1))&amp;MID($B$46,2,999)</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>support</t>
+          <t>work_intro</t>
         </is>
       </c>
       <c r="B48" s="10">
-        <f>IF(OR($B$20="",$B$51),"",", released in support of "&amp;$B$20)</f>
+        <f>IF($B$14=1,$B$11&amp;", ","")&amp;$B$13&amp;IF($B$35="","",IF(LEFT($B$35,1)=",",""," ")&amp;$B$35)</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="B49" s="10">
+        <f>IF(OR($B$20="",$B$52),"",", released in support of "&amp;$B$20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
           <t>beneficiary_tagged</t>
         </is>
       </c>
-      <c r="B49" s="10">
+      <c r="B50" s="10">
         <f>IF($B$20="","",$B$20&amp;IF($B$21="",""," (@"&amp;$B$21&amp;")"))</f>
         <v/>
       </c>
     </row>
-    <row r="50" ht="80" customHeight="1">
-      <c r="A50" s="4" t="inlineStr">
+    <row r="51" ht="80" customHeight="1">
+      <c r="A51" s="4" t="inlineStr">
         <is>
           <t>bio_tagged</t>
         </is>
       </c>
-      <c r="B50" s="10">
-        <f>IF($B$6="",$B$33,SUBSTITUTE($B$33,$B$4,$B$39,1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>hook_names_beneficiary</t>
-        </is>
-      </c>
       <c r="B51" s="10">
-        <f>IF($B$20="",FALSE,ISNUMBER(SEARCH($B$20,$B$34)))</f>
+        <f>IF($B$6="",$B$33,SUBSTITUTE($B$33,$B$4,$B$40,1))</f>
         <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
+          <t>hook_names_beneficiary</t>
+        </is>
+      </c>
+      <c r="B52" s="10">
+        <f>IF($B$20="",FALSE,ISNUMBER(SEARCH($B$20,$B$34)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
           <t>features</t>
         </is>
       </c>
-      <c r="B52" s="10">
+      <c r="B53" s="10">
         <f>$B$26&amp;IF($B$27="","",". "&amp;$B$27)&amp;IF($B$28="","",". "&amp;$B$28)&amp;IF($B$29="","",". "&amp;$B$29)&amp;IF($B$30="","",". "&amp;$B$30)&amp;"."</f>
         <v/>
       </c>
     </row>
-    <row r="53" ht="60" customHeight="1">
-      <c r="A53" s="4" t="inlineStr">
+    <row r="54" ht="60" customHeight="1">
+      <c r="A54" s="4" t="inlineStr">
         <is>
           <t>features_list</t>
         </is>
       </c>
-      <c r="B53" s="10">
+      <c r="B54" s="10">
         <f>"· "&amp;$B$26&amp;IF($B$27="","",CHAR(10)&amp;"· "&amp;$B$27)&amp;IF($B$28="","",CHAR(10)&amp;"· "&amp;$B$28)&amp;IF($B$29="","",CHAR(10)&amp;"· "&amp;$B$29)&amp;IF($B$30="","",CHAR(10)&amp;"· "&amp;$B$30)</f>
         <v/>
       </c>
     </row>
-    <row r="54" ht="70" customHeight="1">
-      <c r="A54" s="4" t="inlineStr">
+    <row r="55" ht="70" customHeight="1">
+      <c r="A55" s="4" t="inlineStr">
         <is>
           <t>features_list_support</t>
         </is>
       </c>
-      <c r="B54" s="10">
-        <f>$B$53&amp;IF(OR($B$20="",$B$51),"",CHAR(10)&amp;"· Released in support of "&amp;$B$20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="4" t="inlineStr">
-        <is>
-          <t>making_ours</t>
-        </is>
-      </c>
       <c r="B55" s="10">
-        <f>SUBSTITUTE($B$35,"printmakers at Make-Ready","our printmakers at Make-Ready")</f>
+        <f>$B$54&amp;IF(OR($B$20="",$B$52),"",CHAR(10)&amp;"· Released in support of "&amp;$B$20)</f>
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>making_ours_tagged</t>
+          <t>making_ours</t>
         </is>
       </c>
       <c r="B56" s="10">
-        <f>SUBSTITUTE($B$35,"printmakers at Make-Ready","our printmakers at Make-Ready (@make__ready)")</f>
+        <f>SUBSTITUTE($B$36,"printmakers at Make-Ready","our printmakers at Make-Ready")</f>
         <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>launch_date</t>
+          <t>making_ours_tagged</t>
         </is>
       </c>
       <c r="B57" s="10">
-        <f>TEXT($B$18,"d mmmm")</f>
+        <f>SUBSTITUTE($B$36,"printmakers at Make-Ready","our printmakers at Make-Ready (@make__ready)")</f>
         <v/>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>launch_time</t>
+          <t>launch_date</t>
         </is>
       </c>
       <c r="B58" s="10">
-        <f>TEXT($B$18,"hh:mm")&amp;" UK time"</f>
+        <f>TEXT($B$18,"d mmmm")</f>
         <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>launch_weekday</t>
+          <t>launch_time</t>
         </is>
       </c>
       <c r="B59" s="10">
-        <f>TEXT($B$18,"dddd")</f>
+        <f>TEXT($B$18,"hh:mm")&amp;" UK time"</f>
         <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>launch_date_dd</t>
+          <t>launch_weekday</t>
         </is>
       </c>
       <c r="B60" s="10">
-        <f>TEXT($B$18,"dd mmmm")</f>
+        <f>TEXT($B$18,"dddd")</f>
         <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>close_date</t>
+          <t>launch_date_dd</t>
         </is>
       </c>
       <c r="B61" s="10">
-        <f>TEXT($B$19,"d mmmm")</f>
+        <f>TEXT($B$18,"dd mmmm")</f>
         <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>close_time</t>
+          <t>close_date</t>
         </is>
       </c>
       <c r="B62" s="10">
-        <f>TEXT($B$19,"hh:mm")&amp;" UK time"</f>
+        <f>TEXT($B$19,"d mmmm")</f>
         <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>close_weekday</t>
+          <t>close_time</t>
         </is>
       </c>
       <c r="B63" s="10">
-        <f>TEXT($B$19,"dddd")</f>
+        <f>TEXT($B$19,"hh:mm")&amp;" UK time"</f>
         <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>close_date_dd</t>
+          <t>close_weekday</t>
         </is>
       </c>
       <c r="B64" s="10">
-        <f>TEXT($B$19,"dd mmmm")</f>
+        <f>TEXT($B$19,"dddd")</f>
         <v/>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>collect_phrase</t>
+          <t>close_date_dd</t>
         </is>
       </c>
       <c r="B65" s="10">
-        <f>SUBSTITUTE($B$13," new "," ",1)</f>
+        <f>TEXT($B$19,"dd mmmm")</f>
         <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>edition_phrase_cap</t>
+          <t>collect_phrase</t>
         </is>
       </c>
       <c r="B66" s="10">
-        <f>UPPER(LEFT($B$13,1))&amp;MID($B$13,2,999)</f>
+        <f>SUBSTITUTE($B$13," new "," ",1)</f>
         <v/>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>window_cap</t>
+          <t>edition_phrase_cap</t>
         </is>
       </c>
       <c r="B67" s="10">
-        <f>UPPER(LEFT($B$17,1))&amp;MID($B$17,2,999)</f>
+        <f>UPPER(LEFT($B$13,1))&amp;MID($B$13,2,999)</f>
         <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>card_line</t>
+          <t>window_cap</t>
         </is>
       </c>
       <c r="B68" s="10">
-        <f>$B$66&amp;" by "&amp;$B$4&amp;"."</f>
+        <f>UPPER(LEFT($B$17,1))&amp;MID($B$17,2,999)</f>
         <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>card_line</t>
         </is>
       </c>
       <c r="B69" s="10">
-        <f>IF($B$12="yes","Untitled",$B$11)&amp;CHAR(10)&amp;$B$68</f>
+        <f>$B$67&amp;" by "&amp;$B$4&amp;"."</f>
         <v/>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>quote_line</t>
+          <t>card</t>
         </is>
       </c>
       <c r="B70" s="10">
-        <f>IF($B$36="","","“"&amp;$B$36&amp;"” – "&amp;$B$4)</f>
+        <f>IF($B$12="yes","Untitled",$B$11)&amp;CHAR(10)&amp;$B$69</f>
         <v/>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>each_artwork</t>
+          <t>quote_line</t>
         </is>
       </c>
       <c r="B71" s="10">
-        <f>IF($B$14&gt;1," for each artwork","")</f>
+        <f>IF($B$37="","","“"&amp;$B$37&amp;"” – "&amp;$B$4)</f>
         <v/>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>work_word</t>
+          <t>each_artwork</t>
         </is>
       </c>
       <c r="B72" s="10">
-        <f>IF($B$14&gt;1,"works","work")</f>
+        <f>IF($B$14&gt;1," for each artwork","")</f>
         <v/>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
+          <t>work_word</t>
+        </is>
+      </c>
+      <c r="B73" s="10">
+        <f>IF($B$14&gt;1,"works","work")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
           <t>add_what</t>
         </is>
       </c>
-      <c r="B73" s="10">
-        <f>IF($B$14&gt;1,$B$42,$B$45)</f>
+      <c r="B74" s="10">
+        <f>IF($B$14&gt;1,$B$43,$B$46)</f>
         <v/>
       </c>
     </row>
@@ -1506,7 +1523,7 @@
         </is>
       </c>
       <c r="C6" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6,"{named}",Inputs!$B$39),"{work}",Inputs!$B$43),"{edition_phrase}",Inputs!$B$13)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6,"{named}",Inputs!$B$40),"{work}",Inputs!$B$44),"{edition_phrase}",Inputs!$B$13)</f>
         <v/>
       </c>
     </row>
@@ -1522,7 +1539,7 @@
         </is>
       </c>
       <c r="C7" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7,"{named}",Inputs!$B$39),"{work}",Inputs!$B$43),"{edition_phrase}",Inputs!$B$13)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7,"{named}",Inputs!$B$40),"{work}",Inputs!$B$44),"{edition_phrase}",Inputs!$B$13)</f>
         <v/>
       </c>
     </row>
@@ -1538,7 +1555,7 @@
         </is>
       </c>
       <c r="C8" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B8,"{named}",Inputs!$B$39),"{work}",Inputs!$B$43),"{edition_phrase}",Inputs!$B$13)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B8,"{named}",Inputs!$B$40),"{work}",Inputs!$B$44),"{edition_phrase}",Inputs!$B$13)</f>
         <v/>
       </c>
     </row>
@@ -1554,7 +1571,7 @@
         </is>
       </c>
       <c r="C9" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B9,"{artist}",Inputs!$B$4),"{quote}",Inputs!$B$36)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B9,"{artist}",Inputs!$B$4),"{quote}",Inputs!$B$37)</f>
         <v/>
       </c>
     </row>
@@ -1570,7 +1587,7 @@
         </is>
       </c>
       <c r="C10" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B10,"{named}",Inputs!$B$39),"{Work}",Inputs!$B$44),"{edition_phrase}",Inputs!$B$13)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B10,"{named}",Inputs!$B$40),"{Work}",Inputs!$B$45),"{edition_phrase}",Inputs!$B$13)</f>
         <v/>
       </c>
     </row>
@@ -1586,7 +1603,7 @@
         </is>
       </c>
       <c r="C11" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B11,"{named}",Inputs!$B$39),"{Work}",Inputs!$B$44),"{window}",Inputs!$B$17)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B11,"{named}",Inputs!$B$40),"{Work}",Inputs!$B$45),"{window}",Inputs!$B$17)</f>
         <v/>
       </c>
     </row>
@@ -1602,7 +1619,7 @@
         </is>
       </c>
       <c r="C12" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B12,"{named}",Inputs!$B$39),"{work}",Inputs!$B$43)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B12,"{named}",Inputs!$B$40),"{work}",Inputs!$B$44)</f>
         <v/>
       </c>
     </row>
@@ -1618,7 +1635,7 @@
         </is>
       </c>
       <c r="C13" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B13,"{named}",Inputs!$B$39),"{work}",Inputs!$B$43)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B13,"{named}",Inputs!$B$40),"{work}",Inputs!$B$44)</f>
         <v/>
       </c>
     </row>
@@ -1634,7 +1651,7 @@
         </is>
       </c>
       <c r="C14" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B14,"{named}",Inputs!$B$39),"{work}",Inputs!$B$43)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B14,"{named}",Inputs!$B$40),"{work}",Inputs!$B$44)</f>
         <v/>
       </c>
     </row>
@@ -1650,7 +1667,7 @@
         </is>
       </c>
       <c r="C15" s="10">
-        <f>SUBSTITUTE(B15,"{features}",Inputs!$B$52)</f>
+        <f>SUBSTITUTE(B15,"{features}",Inputs!$B$53)</f>
         <v/>
       </c>
     </row>
@@ -1666,7 +1683,7 @@
         </is>
       </c>
       <c r="C16" s="10">
-        <f>SUBSTITUTE(B16,"{beneficiary_tagged}",Inputs!$B$49)</f>
+        <f>SUBSTITUTE(B16,"{beneficiary_tagged}",Inputs!$B$50)</f>
         <v/>
       </c>
     </row>
@@ -1682,7 +1699,7 @@
         </is>
       </c>
       <c r="C17" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B17,"{window}",Inputs!$B$17),"{launch_date}",Inputs!$B$57),"{launch_time}",Inputs!$B$58)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B17,"{window}",Inputs!$B$17),"{launch_date}",Inputs!$B$58),"{launch_time}",Inputs!$B$59)</f>
         <v/>
       </c>
     </row>
@@ -1698,7 +1715,7 @@
         </is>
       </c>
       <c r="C18" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B18,"{close_date}",Inputs!$B$61),"{close_time}",Inputs!$B$62)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B18,"{close_date}",Inputs!$B$62),"{close_time}",Inputs!$B$63)</f>
         <v/>
       </c>
     </row>
@@ -1714,7 +1731,7 @@
         </is>
       </c>
       <c r="C19" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B19,"{a_unit}",Inputs!$B$42),"{close_date}",Inputs!$B$61),"{close_time}",Inputs!$B$62)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B19,"{a_unit}",Inputs!$B$43),"{close_date}",Inputs!$B$62),"{close_time}",Inputs!$B$63)</f>
         <v/>
       </c>
     </row>
@@ -1730,7 +1747,7 @@
         </is>
       </c>
       <c r="C20" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B20,"{close_date}",Inputs!$B$61),"{close_time}",Inputs!$B$62)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B20,"{close_date}",Inputs!$B$62),"{close_time}",Inputs!$B$63)</f>
         <v/>
       </c>
     </row>
@@ -1785,7 +1802,7 @@
         </is>
       </c>
       <c r="C24" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B24,"{collab_x}",Inputs!$B$41),"{ordinal}",Inputs!$B$10)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B24,"{collab_x}",Inputs!$B$42),"{ordinal}",Inputs!$B$10)</f>
         <v/>
       </c>
     </row>
@@ -1833,7 +1850,7 @@
         </is>
       </c>
       <c r="C27" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B27,"{link}",Inputs!$B$8),"{window}",Inputs!$B$17),"{launch_date}",Inputs!$B$57),"{launch_time}",Inputs!$B$58)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B27,"{link}",Inputs!$B$8),"{window}",Inputs!$B$17),"{launch_date}",Inputs!$B$58),"{launch_time}",Inputs!$B$59)</f>
         <v/>
       </c>
     </row>
@@ -1849,7 +1866,7 @@
         </is>
       </c>
       <c r="C28" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B28,"{link}",Inputs!$B$8),"{close_date}",Inputs!$B$61),"{close_time}",Inputs!$B$62)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B28,"{link}",Inputs!$B$8),"{close_date}",Inputs!$B$62),"{close_time}",Inputs!$B$63)</f>
         <v/>
       </c>
     </row>
@@ -1865,7 +1882,7 @@
         </is>
       </c>
       <c r="C29" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B29,"{link}",Inputs!$B$8),"{a_unit}",Inputs!$B$42),"{close_date}",Inputs!$B$61),"{close_time}",Inputs!$B$62)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B29,"{link}",Inputs!$B$8),"{a_unit}",Inputs!$B$43),"{close_date}",Inputs!$B$62),"{close_time}",Inputs!$B$63)</f>
         <v/>
       </c>
     </row>
@@ -1920,7 +1937,7 @@
         </is>
       </c>
       <c r="C33" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B33,"{close_date}",Inputs!$B$61),"{close_time}",Inputs!$B$62)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B33,"{close_date}",Inputs!$B$62),"{close_time}",Inputs!$B$63)</f>
         <v/>
       </c>
     </row>
@@ -1952,7 +1969,7 @@
         </is>
       </c>
       <c r="C35" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B35,"{artist}",Inputs!$B$4),"{a_unit}",Inputs!$B$42)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B35,"{artist}",Inputs!$B$4),"{a_unit}",Inputs!$B$43)</f>
         <v/>
       </c>
     </row>
@@ -2007,7 +2024,7 @@
         </is>
       </c>
       <c r="C39" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B39,"{artist}",Inputs!$B$4),"{edition_phrase_cap}",Inputs!$B$66)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B39,"{artist}",Inputs!$B$4),"{edition_phrase_cap}",Inputs!$B$67)</f>
         <v/>
       </c>
     </row>
@@ -2023,7 +2040,7 @@
         </is>
       </c>
       <c r="C40" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B40,"{collab_with}",Inputs!$B$5),"{work_intro}",Inputs!$B$47),"{support}",Inputs!$B$48),"{ordinal}",Inputs!$B$10)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B40,"{collab_with}",Inputs!$B$5),"{work_intro}",Inputs!$B$48),"{support}",Inputs!$B$49),"{ordinal}",Inputs!$B$10)</f>
         <v/>
       </c>
     </row>
@@ -2039,7 +2056,7 @@
         </is>
       </c>
       <c r="C41" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B41,"{window}",Inputs!$B$17),"{launch_time}",Inputs!$B$58),"{launch_weekday}",Inputs!$B$59),"{launch_date_dd}",Inputs!$B$60)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B41,"{window}",Inputs!$B$17),"{launch_time}",Inputs!$B$59),"{launch_weekday}",Inputs!$B$60),"{launch_date_dd}",Inputs!$B$61)</f>
         <v/>
       </c>
     </row>
@@ -2149,7 +2166,7 @@
         </is>
       </c>
       <c r="C49" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B49,"{collab_with}",Inputs!$B$5),"{ordinal}",Inputs!$B$10),"{window}",Inputs!$B$17),"{launch_time}",Inputs!$B$58)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B49,"{collab_with}",Inputs!$B$5),"{ordinal}",Inputs!$B$10),"{window}",Inputs!$B$17),"{launch_time}",Inputs!$B$59)</f>
         <v/>
       </c>
     </row>
@@ -2213,7 +2230,7 @@
         </is>
       </c>
       <c r="C53" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B53,"{collab_with}",Inputs!$B$5),"{work_intro}",Inputs!$B$47),"{support}",Inputs!$B$48),"{ordinal}",Inputs!$B$10)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B53,"{collab_with}",Inputs!$B$5),"{work_intro}",Inputs!$B$48),"{support}",Inputs!$B$49),"{ordinal}",Inputs!$B$10)</f>
         <v/>
       </c>
     </row>
@@ -2229,7 +2246,7 @@
         </is>
       </c>
       <c r="C54" s="10">
-        <f>SUBSTITUTE(B54,"{launch_date}",Inputs!$B$57)</f>
+        <f>SUBSTITUTE(B54,"{launch_date}",Inputs!$B$58)</f>
         <v/>
       </c>
     </row>
@@ -2261,7 +2278,7 @@
         </is>
       </c>
       <c r="C56" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B56,"{collab_with}",Inputs!$B$5),"{work_intro}",Inputs!$B$47),"{support}",Inputs!$B$48),"{ordinal}",Inputs!$B$10)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B56,"{collab_with}",Inputs!$B$5),"{work_intro}",Inputs!$B$48),"{support}",Inputs!$B$49),"{ordinal}",Inputs!$B$10)</f>
         <v/>
       </c>
     </row>
@@ -2277,7 +2294,7 @@
         </is>
       </c>
       <c r="C57" s="10">
-        <f>SUBSTITUTE(B57,"{launch_date}",Inputs!$B$57)</f>
+        <f>SUBSTITUTE(B57,"{launch_date}",Inputs!$B$58)</f>
         <v/>
       </c>
     </row>
@@ -2293,7 +2310,7 @@
         </is>
       </c>
       <c r="C58" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B58,"{window}",Inputs!$B$17),"{launch_time}",Inputs!$B$58)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B58,"{window}",Inputs!$B$17),"{launch_time}",Inputs!$B$59)</f>
         <v/>
       </c>
     </row>
@@ -2366,7 +2383,7 @@
         </is>
       </c>
       <c r="C63" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B63,"{collab_with}",Inputs!$B$5),"{work_intro}",Inputs!$B$47),"{support}",Inputs!$B$48),"{ordinal}",Inputs!$B$10),"{window}",Inputs!$B$17)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B63,"{collab_with}",Inputs!$B$5),"{work_intro}",Inputs!$B$48),"{support}",Inputs!$B$49),"{ordinal}",Inputs!$B$10),"{window}",Inputs!$B$17)</f>
         <v/>
       </c>
     </row>
@@ -2382,7 +2399,7 @@
         </is>
       </c>
       <c r="C64" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B64,"{close_time}",Inputs!$B$62),"{close_weekday}",Inputs!$B$63),"{close_date_dd}",Inputs!$B$64),"{add_what}",Inputs!$B$73)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B64,"{close_time}",Inputs!$B$63),"{close_weekday}",Inputs!$B$64),"{close_date_dd}",Inputs!$B$65),"{add_what}",Inputs!$B$74)</f>
         <v/>
       </c>
     </row>
@@ -2414,7 +2431,7 @@
         </is>
       </c>
       <c r="C66" s="10">
-        <f>SUBSTITUTE(B66,"{a_unit}",Inputs!$B$42)</f>
+        <f>SUBSTITUTE(B66,"{a_unit}",Inputs!$B$43)</f>
         <v/>
       </c>
     </row>
@@ -2462,7 +2479,7 @@
         </is>
       </c>
       <c r="C69" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B69,"{artist}",Inputs!$B$4),"{collect_phrase}",Inputs!$B$65)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B69,"{artist}",Inputs!$B$4),"{collect_phrase}",Inputs!$B$66)</f>
         <v/>
       </c>
     </row>
@@ -2478,7 +2495,7 @@
         </is>
       </c>
       <c r="C70" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B70,"{close_time}",Inputs!$B$62),"{close_weekday}",Inputs!$B$63),"{close_date_dd}",Inputs!$B$64)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B70,"{close_time}",Inputs!$B$63),"{close_weekday}",Inputs!$B$64),"{close_date_dd}",Inputs!$B$65)</f>
         <v/>
       </c>
     </row>
@@ -2494,7 +2511,7 @@
         </is>
       </c>
       <c r="C71" s="10">
-        <f>SUBSTITUTE(B71,"{a_unit}",Inputs!$B$42)</f>
+        <f>SUBSTITUTE(B71,"{a_unit}",Inputs!$B$43)</f>
         <v/>
       </c>
     </row>
@@ -2517,7 +2534,7 @@
         </is>
       </c>
       <c r="C73" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B73,"{collab_with}",Inputs!$B$5),"{collect_phrase}",Inputs!$B$65),"{ordinal}",Inputs!$B$10),"{close_time}",Inputs!$B$62),"{close_weekday}",Inputs!$B$63),"{close_date_dd}",Inputs!$B$64)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B73,"{collab_with}",Inputs!$B$5),"{collect_phrase}",Inputs!$B$66),"{ordinal}",Inputs!$B$10),"{close_time}",Inputs!$B$63),"{close_weekday}",Inputs!$B$64),"{close_date_dd}",Inputs!$B$65)</f>
         <v/>
       </c>
     </row>
@@ -2533,7 +2550,7 @@
         </is>
       </c>
       <c r="C74" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B74,"{each_artwork}",Inputs!$B$71),"{work_word}",Inputs!$B$72)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B74,"{each_artwork}",Inputs!$B$72),"{work_word}",Inputs!$B$73)</f>
         <v/>
       </c>
     </row>
@@ -2549,7 +2566,7 @@
         </is>
       </c>
       <c r="C75" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B75,"{artist}",Inputs!$B$4),"{work_email}",Inputs!$B$45),"{collect_phrase}",Inputs!$B$65)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B75,"{artist}",Inputs!$B$4),"{work_email}",Inputs!$B$46),"{collect_phrase}",Inputs!$B$66)</f>
         <v/>
       </c>
     </row>
@@ -2565,7 +2582,7 @@
         </is>
       </c>
       <c r="C76" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B76,"{close_time}",Inputs!$B$62),"{close_weekday}",Inputs!$B$63),"{close_date_dd}",Inputs!$B$64)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B76,"{close_time}",Inputs!$B$63),"{close_weekday}",Inputs!$B$64),"{close_date_dd}",Inputs!$B$65)</f>
         <v/>
       </c>
     </row>
@@ -2755,7 +2772,7 @@
         </is>
       </c>
       <c r="C89" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B89,"{collab_with}",Inputs!$B$5),"{work_intro}",Inputs!$B$47),"{support}",Inputs!$B$48)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B89,"{collab_with}",Inputs!$B$5),"{work_intro}",Inputs!$B$48),"{support}",Inputs!$B$49)</f>
         <v/>
       </c>
     </row>
@@ -2771,7 +2788,7 @@
         </is>
       </c>
       <c r="C90" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B90,"{close_date}",Inputs!$B$61),"{close_time}",Inputs!$B$62)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B90,"{close_date}",Inputs!$B$62),"{close_time}",Inputs!$B$63)</f>
         <v/>
       </c>
     </row>
@@ -2787,7 +2804,7 @@
         </is>
       </c>
       <c r="C91" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B91,"{window}",Inputs!$B$17),"{launch_time}",Inputs!$B$58),"{launch_weekday}",Inputs!$B$59),"{launch_date_dd}",Inputs!$B$60)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B91,"{window}",Inputs!$B$17),"{launch_time}",Inputs!$B$59),"{launch_weekday}",Inputs!$B$60),"{launch_date_dd}",Inputs!$B$61)</f>
         <v/>
       </c>
     </row>
@@ -2913,7 +2930,7 @@
         <v/>
       </c>
       <c r="F4" s="11">
-        <f>Inputs!$B$50</f>
+        <f>Inputs!$B$51</f>
         <v/>
       </c>
       <c r="G4" s="11">
@@ -2965,7 +2982,7 @@
         <v/>
       </c>
       <c r="G5" s="11">
-        <f>Lines!$C$15&amp;IF(Inputs!$B$51,"",IF(Inputs!$B$49="",""," "&amp;Lines!$C$16))</f>
+        <f>Lines!$C$15&amp;IF(Inputs!$B$52,"",IF(Inputs!$B$50="",""," "&amp;Lines!$C$16))</f>
         <v/>
       </c>
       <c r="H5" s="11">
@@ -3009,11 +3026,11 @@
         <v/>
       </c>
       <c r="F6" s="11">
-        <f>Inputs!$B$56</f>
+        <f>Inputs!$B$57</f>
         <v/>
       </c>
       <c r="G6" s="11">
-        <f>Lines!$C$15&amp;IF(Inputs!$B$49="",""," "&amp;Lines!$C$16)</f>
+        <f>Lines!$C$15&amp;IF(Inputs!$B$50="",""," "&amp;Lines!$C$16)</f>
         <v/>
       </c>
       <c r="H6" s="11">
@@ -3053,19 +3070,19 @@
         </is>
       </c>
       <c r="E7" s="11">
-        <f>IF(Inputs!$B$36="","(no quote given, post skipped)",Lines!$C$9)</f>
+        <f>IF(Inputs!$B$37="","(no quote given, post skipped)",Lines!$C$9)</f>
         <v/>
       </c>
       <c r="F7" s="11">
-        <f>IF(Inputs!$B$36="","",Lines!$C$10)</f>
+        <f>IF(Inputs!$B$37="","",Lines!$C$10)</f>
         <v/>
       </c>
       <c r="G7" s="11">
-        <f>IF(Inputs!$B$36="","",Lines!$C$15&amp;IF(Inputs!$B$49="",""," "&amp;Lines!$C$16))</f>
+        <f>IF(Inputs!$B$37="","",Lines!$C$15&amp;IF(Inputs!$B$50="",""," "&amp;Lines!$C$16))</f>
         <v/>
       </c>
       <c r="H7" s="11">
-        <f>IF(Inputs!$B$36="","",IF(Inputs!$B$16="draw",Lines!$C$18,Lines!$C$17))</f>
+        <f>IF(Inputs!$B$37="","",IF(Inputs!$B$16="draw",Lines!$C$18,Lines!$C$17))</f>
         <v/>
       </c>
       <c r="I7" s="11">
@@ -3073,7 +3090,7 @@
         <v/>
       </c>
       <c r="J7" s="11">
-        <f>IF(Inputs!$B$36="","(no quote given, post skipped)",E7&amp;IF(F7="","",CHAR(10)&amp;CHAR(10)&amp;F7)&amp;IF(G7="","",CHAR(10)&amp;CHAR(10)&amp;G7)&amp;IF(H7="","",CHAR(10)&amp;CHAR(10)&amp;H7))</f>
+        <f>IF(Inputs!$B$37="","(no quote given, post skipped)",E7&amp;IF(F7="","",CHAR(10)&amp;CHAR(10)&amp;F7)&amp;IF(G7="","",CHAR(10)&amp;CHAR(10)&amp;G7)&amp;IF(H7="","",CHAR(10)&amp;CHAR(10)&amp;H7))</f>
         <v/>
       </c>
       <c r="K7" s="11">
@@ -3109,7 +3126,7 @@
         <v/>
       </c>
       <c r="G8" s="11">
-        <f>IF(Inputs!$B$16="draw","",Lines!$C$15&amp;IF(Inputs!$B$49="",""," "&amp;Lines!$C$16))</f>
+        <f>IF(Inputs!$B$16="draw","",Lines!$C$15&amp;IF(Inputs!$B$50="",""," "&amp;Lines!$C$16))</f>
         <v/>
       </c>
       <c r="H8" s="11">
@@ -3157,7 +3174,7 @@
         <v/>
       </c>
       <c r="G9" s="11">
-        <f>IF(Inputs!$B$16="draw","",Lines!$C$15&amp;IF(Inputs!$B$49="",""," "&amp;Lines!$C$16))</f>
+        <f>IF(Inputs!$B$16="draw","",Lines!$C$15&amp;IF(Inputs!$B$50="",""," "&amp;Lines!$C$16))</f>
         <v/>
       </c>
       <c r="H9" s="11">
@@ -3205,7 +3222,7 @@
         <v/>
       </c>
       <c r="G10" s="11">
-        <f>Lines!$C$15&amp;IF(Inputs!$B$49="",""," "&amp;Lines!$C$16)</f>
+        <f>Lines!$C$15&amp;IF(Inputs!$B$50="",""," "&amp;Lines!$C$16)</f>
         <v/>
       </c>
       <c r="H10" s="11">
@@ -3365,7 +3382,7 @@
         </is>
       </c>
       <c r="D5" s="11">
-        <f>SUBSTITUTE(IF(Inputs!$B$12="yes",Lines!$C$7,Lines!$C$6),Inputs!$B$39,Inputs!$B$40)</f>
+        <f>SUBSTITUTE(IF(Inputs!$B$12="yes",Lines!$C$7,Lines!$C$6),Inputs!$B$40,Inputs!$B$41)</f>
         <v/>
       </c>
       <c r="E5" s="11">
@@ -3373,7 +3390,7 @@
         <v/>
       </c>
       <c r="F5" s="11">
-        <f>IF(OR(Inputs!$B$20="",Inputs!$B$51),"",Lines!$C$26)</f>
+        <f>IF(OR(Inputs!$B$20="",Inputs!$B$52),"",Lines!$C$26)</f>
         <v/>
       </c>
       <c r="G5" s="11">
@@ -3404,7 +3421,7 @@
         </is>
       </c>
       <c r="D6" s="11">
-        <f>IF(Inputs!$B$16="draw","(not used for a draw)",SUBSTITUTE(Lines!$C$11,Inputs!$B$39,Inputs!$B$40))</f>
+        <f>IF(Inputs!$B$16="draw","(not used for a draw)",SUBSTITUTE(Lines!$C$11,Inputs!$B$40,Inputs!$B$41))</f>
         <v/>
       </c>
       <c r="E6" s="11">
@@ -3443,7 +3460,7 @@
         </is>
       </c>
       <c r="D7" s="11">
-        <f>IF(Inputs!$B$16="draw","(not used for a draw)",SUBSTITUTE(Lines!$C$12,Inputs!$B$39,Inputs!$B$40))</f>
+        <f>IF(Inputs!$B$16="draw","(not used for a draw)",SUBSTITUTE(Lines!$C$12,Inputs!$B$40,Inputs!$B$41))</f>
         <v/>
       </c>
       <c r="E7" s="11">
@@ -3482,7 +3499,7 @@
         </is>
       </c>
       <c r="D8" s="11">
-        <f>IF(Inputs!$B$16="draw",SUBSTITUTE(Lines!$C$14,Inputs!$B$39,Inputs!$B$40),SUBSTITUTE(Lines!$C$13,Inputs!$B$39,Inputs!$B$40))</f>
+        <f>IF(Inputs!$B$16="draw",SUBSTITUTE(Lines!$C$14,Inputs!$B$40,Inputs!$B$41),SUBSTITUTE(Lines!$C$13,Inputs!$B$40,Inputs!$B$41))</f>
         <v/>
       </c>
       <c r="E8" s="11">
@@ -3651,19 +3668,19 @@
         <v/>
       </c>
       <c r="F4" s="11">
-        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$16="draw","Enter the draw for a chance to collect. Closes "&amp;Inputs!$B$61&amp;".","Launching "&amp;Inputs!$B$57&amp;". Register for updates."))</f>
+        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$16="draw","Enter the draw for a chance to collect. Closes "&amp;Inputs!$B$62&amp;".","Launching "&amp;Inputs!$B$58&amp;". Register for updates."))</f>
         <v/>
       </c>
       <c r="G4" s="11">
-        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$16="draw","Enter the draw","Launching "&amp;Inputs!$B$57))</f>
+        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$16="draw","Enter the draw","Launching "&amp;Inputs!$B$58))</f>
         <v/>
       </c>
       <c r="H4" s="11">
-        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$16="draw",Inputs!$B$46,Inputs!$B$46&amp;" by "&amp;Inputs!$B$4))</f>
+        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$16="draw",Inputs!$B$47,Inputs!$B$47&amp;" by "&amp;Inputs!$B$4))</f>
         <v/>
       </c>
       <c r="I4" s="11">
-        <f>IF($D4&lt;&gt;"yes","",(Lines!$C$40&amp;IF(Inputs!$B$34="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$34)&amp;IF(Inputs!$B$55="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$55)&amp;IF(Inputs!$B$53="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$53)&amp;IF(IF(Inputs!$B$16="draw",Lines!$C$33,(Lines!$C$41&amp;IF(Lines!$C$42="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$42)))="","",CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$16="draw",Lines!$C$33,(Lines!$C$41&amp;IF(Lines!$C$42="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$42))))))</f>
+        <f>IF($D4&lt;&gt;"yes","",(Lines!$C$40&amp;IF(Inputs!$B$34="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$34)&amp;IF(Inputs!$B$56="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$56)&amp;IF(Inputs!$B$54="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$54)&amp;IF(IF(Inputs!$B$16="draw",Lines!$C$33,(Lines!$C$41&amp;IF(Lines!$C$42="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$42)))="","",CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$16="draw",Lines!$C$33,(Lines!$C$41&amp;IF(Lines!$C$42="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$42))))))</f>
         <v/>
       </c>
       <c r="J4" s="11">
@@ -3671,15 +3688,15 @@
         <v/>
       </c>
       <c r="K4" s="11">
-        <f>IF($D4&lt;&gt;"yes","",Inputs!$B$69)</f>
+        <f>IF($D4&lt;&gt;"yes","",Inputs!$B$70)</f>
         <v/>
       </c>
       <c r="L4" s="11">
-        <f>IF($D4&lt;&gt;"yes","",Inputs!$B$70)</f>
+        <f>IF($D4&lt;&gt;"yes","",Inputs!$B$71)</f>
         <v/>
       </c>
       <c r="M4" s="11">
-        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$16="draw","Collect "&amp;Inputs!$B$65,"Launching "&amp;Inputs!$B$57))</f>
+        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$16="draw","Collect "&amp;Inputs!$B$66,"Launching "&amp;Inputs!$B$58))</f>
         <v/>
       </c>
       <c r="N4" s="11">
@@ -3789,7 +3806,7 @@
         <v/>
       </c>
       <c r="I6" s="11">
-        <f>IF($D6&lt;&gt;"yes","",(Lines!$C$31&amp;IF(Lines!$C$49="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$49)&amp;IF(Inputs!$B$34="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$34)&amp;IF(Inputs!$B$54="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$54)&amp;IF(Lines!$C$50="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$50)&amp;IF(IF(Inputs!$B$24="","",Lines!$C$36)="","",CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$24="","",Lines!$C$36))&amp;IF(Lines!$C$52="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$52)))</f>
+        <f>IF($D6&lt;&gt;"yes","",(Lines!$C$31&amp;IF(Lines!$C$49="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$49)&amp;IF(Inputs!$B$34="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$34)&amp;IF(Inputs!$B$55="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$55)&amp;IF(Lines!$C$50="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$50)&amp;IF(IF(Inputs!$B$24="","",Lines!$C$36)="","",CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$24="","",Lines!$C$36))&amp;IF(Lines!$C$52="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$52)))</f>
         <v/>
       </c>
       <c r="J6" s="11">
@@ -3852,7 +3869,7 @@
         <v/>
       </c>
       <c r="I7" s="11">
-        <f>IF($D7&lt;&gt;"yes","",(Lines!$C$31&amp;IF(Lines!$C$49="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$49)&amp;IF(Inputs!$B$34="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$34)&amp;IF(Inputs!$B$54="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$54)&amp;IF(Lines!$C$51="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$51)&amp;IF(Lines!$C$52="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$52)&amp;IF(Lines!$C$34="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$34)&amp;IF(Lines!$C$32="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$32)))</f>
+        <f>IF($D7&lt;&gt;"yes","",(Lines!$C$31&amp;IF(Lines!$C$49="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$49)&amp;IF(Inputs!$B$34="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$34)&amp;IF(Inputs!$B$55="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$55)&amp;IF(Lines!$C$51="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$51)&amp;IF(Lines!$C$52="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$52)&amp;IF(Lines!$C$34="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$34)&amp;IF(Lines!$C$32="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$32)))</f>
         <v/>
       </c>
       <c r="J7" s="11">
@@ -3860,7 +3877,7 @@
         <v/>
       </c>
       <c r="K7" s="11">
-        <f>IF($D7&lt;&gt;"yes","",Inputs!$B$69)</f>
+        <f>IF($D7&lt;&gt;"yes","",Inputs!$B$70)</f>
         <v/>
       </c>
       <c r="L7" s="11">
@@ -3923,7 +3940,7 @@
         <v/>
       </c>
       <c r="K8" s="11">
-        <f>IF($D8&lt;&gt;"yes","",Inputs!$B$69)</f>
+        <f>IF($D8&lt;&gt;"yes","",Inputs!$B$70)</f>
         <v/>
       </c>
       <c r="L8" s="11">
@@ -3986,7 +4003,7 @@
         <v/>
       </c>
       <c r="K9" s="11">
-        <f>IF($D9&lt;&gt;"yes","",Inputs!$B$69)</f>
+        <f>IF($D9&lt;&gt;"yes","",Inputs!$B$70)</f>
         <v/>
       </c>
       <c r="L9" s="11">
@@ -4029,7 +4046,7 @@
         <v/>
       </c>
       <c r="F10" s="11">
-        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$67&amp;", starting now.")</f>
+        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$68&amp;", starting now.")</f>
         <v/>
       </c>
       <c r="G10" s="11">
@@ -4037,11 +4054,11 @@
         <v/>
       </c>
       <c r="H10" s="11">
-        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$67&amp;", starting now")</f>
+        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$68&amp;", starting now")</f>
         <v/>
       </c>
       <c r="I10" s="11">
-        <f>IF($D10&lt;&gt;"yes","",(Lines!$C$63&amp;IF(Inputs!$B$34="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$34)&amp;IF(Inputs!$B$55="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$55)&amp;IF(Inputs!$B$54="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$54)&amp;IF(Lines!$C$64="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$64)&amp;IF(IF(Inputs!$B$24="","",Lines!$C$36)="","",CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$24="","",Lines!$C$36))))</f>
+        <f>IF($D10&lt;&gt;"yes","",(Lines!$C$63&amp;IF(Inputs!$B$34="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$34)&amp;IF(Inputs!$B$56="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$56)&amp;IF(Inputs!$B$55="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$55)&amp;IF(Lines!$C$64="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$64)&amp;IF(IF(Inputs!$B$24="","",Lines!$C$36)="","",CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$24="","",Lines!$C$36))))</f>
         <v/>
       </c>
       <c r="J10" s="11">
@@ -4049,15 +4066,15 @@
         <v/>
       </c>
       <c r="K10" s="11">
-        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$69)</f>
+        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$70)</f>
         <v/>
       </c>
       <c r="L10" s="11">
-        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$70)</f>
+        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$71)</f>
         <v/>
       </c>
       <c r="M10" s="11">
-        <f>IF($D10&lt;&gt;"yes","","Collect "&amp;Inputs!$B$65)</f>
+        <f>IF($D10&lt;&gt;"yes","","Collect "&amp;Inputs!$B$66)</f>
         <v/>
       </c>
       <c r="N10" s="11">
@@ -4171,7 +4188,7 @@
         <v/>
       </c>
       <c r="J12" s="11">
-        <f>IF($D12&lt;&gt;"yes","","Buy "&amp;Inputs!$B$42)</f>
+        <f>IF($D12&lt;&gt;"yes","","Buy "&amp;Inputs!$B$43)</f>
         <v/>
       </c>
       <c r="K12" s="11">
@@ -4222,7 +4239,7 @@
         <v/>
       </c>
       <c r="G13" s="11">
-        <f>IF($D13&lt;&gt;"yes","",Inputs!$B$46&amp;" by "&amp;Inputs!$B$4)</f>
+        <f>IF($D13&lt;&gt;"yes","",Inputs!$B$47&amp;" by "&amp;Inputs!$B$4)</f>
         <v/>
       </c>
       <c r="H13" s="11">
@@ -4234,11 +4251,11 @@
         <v/>
       </c>
       <c r="J13" s="11">
-        <f>IF($D13&lt;&gt;"yes","","Buy "&amp;Inputs!$B$42)</f>
+        <f>IF($D13&lt;&gt;"yes","","Buy "&amp;Inputs!$B$43)</f>
         <v/>
       </c>
       <c r="K13" s="11">
-        <f>IF($D13&lt;&gt;"yes","",Inputs!$B$69)</f>
+        <f>IF($D13&lt;&gt;"yes","",Inputs!$B$70)</f>
         <v/>
       </c>
       <c r="L13" s="11">
@@ -4281,7 +4298,7 @@
         <v/>
       </c>
       <c r="F14" s="11">
-        <f>IF($D14&lt;&gt;"yes","",IF(Inputs!$B$16="draw","The draw closes at "&amp;Inputs!$B$62&amp;" on "&amp;Inputs!$B$61&amp;".","Time is almost up."))</f>
+        <f>IF($D14&lt;&gt;"yes","",IF(Inputs!$B$16="draw","The draw closes at "&amp;Inputs!$B$63&amp;" on "&amp;Inputs!$B$62&amp;".","Time is almost up."))</f>
         <v/>
       </c>
       <c r="G14" s="11">
@@ -4301,7 +4318,7 @@
         <v/>
       </c>
       <c r="K14" s="11">
-        <f>IF($D14&lt;&gt;"yes","",Inputs!$B$69)</f>
+        <f>IF($D14&lt;&gt;"yes","",Inputs!$B$70)</f>
         <v/>
       </c>
       <c r="L14" s="11">
@@ -4482,7 +4499,7 @@
         <v/>
       </c>
       <c r="I17" s="11">
-        <f>IF($D17&lt;&gt;"yes","",(Lines!$C$89&amp;IF(Inputs!$B$34="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$34)&amp;IF(Inputs!$B$55="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$55)&amp;IF(IF(Inputs!$B$16="draw",Lines!$C$90,Lines!$C$91)="","",CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$16="draw",Lines!$C$90,Lines!$C$91))))</f>
+        <f>IF($D17&lt;&gt;"yes","",(Lines!$C$89&amp;IF(Inputs!$B$34="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$34)&amp;IF(Inputs!$B$56="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$56)&amp;IF(IF(Inputs!$B$16="draw",Lines!$C$90,Lines!$C$91)="","",CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$16="draw",Lines!$C$90,Lines!$C$91))))</f>
         <v/>
       </c>
       <c r="J17" s="11">
@@ -4603,7 +4620,7 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>The opener names the work only for a single print: 'The Changeling, a new limited edition print'. A pair or a quartet is just the edition phrase, and the hook names the work; many sets have no collective name anyway. Untitled works from a named series read 'six new limited edition prints from the Dream House series'.</t>
+          <t>The opener's tail is the title (single print only), the edition phrase, and the qualifier if one is written: 'The Changeling, a new limited edition print'; 'a quartet of new limited edition prints spanning five decades of the artist's career'; 'six new limited edition prints from his iconic Dream House series'. A pair or a quartet takes no title; the hook names the work. The same tail is used by the Insiders email, LE early access, Now Live and the Monthly Preview paragraph.</t>
         </is>
       </c>
     </row>

</xml_diff>